<commit_message>
Fix excel and add timeouts
</commit_message>
<xml_diff>
--- a/dotabuff_matches_stats.xlsx
+++ b/dotabuff_matches_stats.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G2"/>
+  <dimension ref="A1:G4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -486,7 +486,67 @@
       <c r="F2" t="n">
         <v>10</v>
       </c>
-      <c r="G2" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>8609332493</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>38:30</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>28 - 60</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Dire (Тьма)</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Dire</t>
+        </is>
+      </c>
+      <c r="F3" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>8609356930</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>23:15</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>31 - 6</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Radiant (Светлая)</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Radiant</t>
+        </is>
+      </c>
+      <c r="F4" t="n">
+        <v>10</v>
+      </c>
+      <c r="G4" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -499,7 +559,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q11"/>
+  <dimension ref="A1:Q31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -660,9 +720,6 @@
           <t>17.4k</t>
         </is>
       </c>
-      <c r="O2" t="inlineStr"/>
-      <c r="P2" t="inlineStr"/>
-      <c r="Q2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -735,9 +792,6 @@
           <t>8.2k</t>
         </is>
       </c>
-      <c r="O3" t="inlineStr"/>
-      <c r="P3" t="inlineStr"/>
-      <c r="Q3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -810,9 +864,6 @@
           <t>13.4k</t>
         </is>
       </c>
-      <c r="O4" t="inlineStr"/>
-      <c r="P4" t="inlineStr"/>
-      <c r="Q4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -885,9 +936,6 @@
           <t>9.0k</t>
         </is>
       </c>
-      <c r="O5" t="inlineStr"/>
-      <c r="P5" t="inlineStr"/>
-      <c r="Q5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -960,9 +1008,6 @@
           <t>22.0k</t>
         </is>
       </c>
-      <c r="O6" t="inlineStr"/>
-      <c r="P6" t="inlineStr"/>
-      <c r="Q6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -1035,9 +1080,6 @@
           <t>12.1k</t>
         </is>
       </c>
-      <c r="O7" t="inlineStr"/>
-      <c r="P7" t="inlineStr"/>
-      <c r="Q7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -1110,9 +1152,6 @@
           <t>29.5k</t>
         </is>
       </c>
-      <c r="O8" t="inlineStr"/>
-      <c r="P8" t="inlineStr"/>
-      <c r="Q8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -1185,9 +1224,6 @@
           <t>29.6k</t>
         </is>
       </c>
-      <c r="O9" t="inlineStr"/>
-      <c r="P9" t="inlineStr"/>
-      <c r="Q9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -1260,9 +1296,6 @@
           <t>11.4k</t>
         </is>
       </c>
-      <c r="O10" t="inlineStr"/>
-      <c r="P10" t="inlineStr"/>
-      <c r="Q10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -1335,9 +1368,1464 @@
           <t>24.4k</t>
         </is>
       </c>
-      <c r="O11" t="inlineStr"/>
-      <c r="P11" t="inlineStr"/>
-      <c r="Q11" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>8609332493</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Radiant</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Skywrath Mage</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>средняя линия</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>ключевая роль</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>Shield of the Scion</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>411</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>Shield of the Scion</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>Shield of the Scion</t>
+        </is>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>13</t>
+        </is>
+      </c>
+      <c r="M12" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="N12" t="inlineStr">
+        <is>
+          <t>17.4k</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>8609332493</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Radiant</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Shadow Shaman</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>роль поддержки</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>Chicken Fingers</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>468</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>Chicken Fingers</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>Chicken Fingers</t>
+        </is>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="L13" t="inlineStr">
+        <is>
+          <t>14</t>
+        </is>
+      </c>
+      <c r="M13" t="inlineStr">
+        <is>
+          <t>14</t>
+        </is>
+      </c>
+      <c r="N13" t="inlineStr">
+        <is>
+          <t>8.2k</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>8609332493</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Radiant</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Vengeful Spirit</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>сложная линия</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>ключевая роль</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>Soul Strike</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>5123</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>Soul Strike</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>Soul Strike</t>
+        </is>
+      </c>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="L14" t="inlineStr">
+        <is>
+          <t>13</t>
+        </is>
+      </c>
+      <c r="M14" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="N14" t="inlineStr">
+        <is>
+          <t>13.4k</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>8609332493</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Radiant</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Largo</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>легкая линия</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>роль поддержки</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>Musical pilgrimage</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>1661</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>Musical pilgrimage</t>
+        </is>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>Musical pilgrimage</t>
+        </is>
+      </c>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="L15" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="M15" t="inlineStr">
+        <is>
+          <t>13</t>
+        </is>
+      </c>
+      <c r="N15" t="inlineStr">
+        <is>
+          <t>9.0k</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>8609332493</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Radiant</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Ursa</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>легкая линия</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>ключевая роль</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>Bear Down</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>5358</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>Bear Down</t>
+        </is>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>Bear Down</t>
+        </is>
+      </c>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="L16" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="M16" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="N16" t="inlineStr">
+        <is>
+          <t>22.0k</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>8609332493</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Dire</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Tusk</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>роль поддержки</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>Tag Team</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>5566</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>Tag Team</t>
+        </is>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>Tag Team</t>
+        </is>
+      </c>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="L17" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="M17" t="inlineStr">
+        <is>
+          <t>38</t>
+        </is>
+      </c>
+      <c r="N17" t="inlineStr">
+        <is>
+          <t>12.1k</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>8609332493</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Dire</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Drow Ranger</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>легкая линия</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>ключевая роль</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>Sidestep</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>5019</t>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>Sidestep</t>
+        </is>
+      </c>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>Sidestep</t>
+        </is>
+      </c>
+      <c r="K18" t="inlineStr">
+        <is>
+          <t>21</t>
+        </is>
+      </c>
+      <c r="L18" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="M18" t="inlineStr">
+        <is>
+          <t>21</t>
+        </is>
+      </c>
+      <c r="N18" t="inlineStr">
+        <is>
+          <t>29.5k</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>8609332493</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Dire</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Arc Warden</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>средняя линия</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>ключевая роль</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>Runed Replica</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>7120</t>
+        </is>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>Runed Replica</t>
+        </is>
+      </c>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>Runed Replica</t>
+        </is>
+      </c>
+      <c r="K19" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="L19" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="M19" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+      <c r="N19" t="inlineStr">
+        <is>
+          <t>29.6k</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>8609332493</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Dire</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Lion</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>сложная линия</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>роль поддержки</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>Fist of Death</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>465</t>
+        </is>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>Fist of Death</t>
+        </is>
+      </c>
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>Fist of Death</t>
+        </is>
+      </c>
+      <c r="K20" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="L20" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="M20" t="inlineStr">
+        <is>
+          <t>30</t>
+        </is>
+      </c>
+      <c r="N20" t="inlineStr">
+        <is>
+          <t>11.4k</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>8609332493</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Dire</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Magnus</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>сложная линия</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>ключевая роль</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>Eternal Empowerment</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>5518</t>
+        </is>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>Eternal Empowerment</t>
+        </is>
+      </c>
+      <c r="J21" t="inlineStr">
+        <is>
+          <t>Eternal Empowerment</t>
+        </is>
+      </c>
+      <c r="K21" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="L21" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="M21" t="inlineStr">
+        <is>
+          <t>29</t>
+        </is>
+      </c>
+      <c r="N21" t="inlineStr">
+        <is>
+          <t>24.4k</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>8609356930</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Radiant</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Troll Warlord</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>Bad Influence</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>5508</t>
+        </is>
+      </c>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>Bad Influence</t>
+        </is>
+      </c>
+      <c r="J22" t="inlineStr">
+        <is>
+          <t>Bad Influence</t>
+        </is>
+      </c>
+      <c r="K22" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="L22" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="M22" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="N22" t="inlineStr">
+        <is>
+          <t>15.2k</t>
+        </is>
+      </c>
+      <c r="O22" t="inlineStr"/>
+      <c r="P22" t="inlineStr"/>
+      <c r="Q22" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>8609356930</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Radiant</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Mars</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>Victory Feast</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>1020</t>
+        </is>
+      </c>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>Victory Feast</t>
+        </is>
+      </c>
+      <c r="J23" t="inlineStr">
+        <is>
+          <t>Victory Feast</t>
+        </is>
+      </c>
+      <c r="K23" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="L23" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="M23" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="N23" t="inlineStr">
+        <is>
+          <t>8.8k</t>
+        </is>
+      </c>
+      <c r="O23" t="inlineStr"/>
+      <c r="P23" t="inlineStr"/>
+      <c r="Q23" t="inlineStr"/>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>8609356930</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Radiant</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Pudge</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>Fresh Meat</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>5074</t>
+        </is>
+      </c>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>Fresh Meat</t>
+        </is>
+      </c>
+      <c r="J24" t="inlineStr">
+        <is>
+          <t>Fresh Meat</t>
+        </is>
+      </c>
+      <c r="K24" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="L24" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="M24" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="N24" t="inlineStr">
+        <is>
+          <t>7.5k</t>
+        </is>
+      </c>
+      <c r="O24" t="inlineStr"/>
+      <c r="P24" t="inlineStr"/>
+      <c r="Q24" t="inlineStr"/>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>8609356930</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Radiant</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>Natures Prophet</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>Soothing Saplings</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>470</t>
+        </is>
+      </c>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>Soothing Saplings</t>
+        </is>
+      </c>
+      <c r="J25" t="inlineStr">
+        <is>
+          <t>Soothing Saplings</t>
+        </is>
+      </c>
+      <c r="K25" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="L25" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="M25" t="inlineStr">
+        <is>
+          <t>13</t>
+        </is>
+      </c>
+      <c r="N25" t="inlineStr">
+        <is>
+          <t>12.0k</t>
+        </is>
+      </c>
+      <c r="O25" t="inlineStr"/>
+      <c r="P25" t="inlineStr"/>
+      <c r="Q25" t="inlineStr"/>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>8609356930</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Radiant</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>Hoodwink</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>Go Nuts</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>9501</t>
+        </is>
+      </c>
+      <c r="I26" t="inlineStr">
+        <is>
+          <t>Go Nuts</t>
+        </is>
+      </c>
+      <c r="J26" t="inlineStr">
+        <is>
+          <t>Go Nuts</t>
+        </is>
+      </c>
+      <c r="K26" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="L26" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="M26" t="inlineStr">
+        <is>
+          <t>14</t>
+        </is>
+      </c>
+      <c r="N26" t="inlineStr">
+        <is>
+          <t>7.6k</t>
+        </is>
+      </c>
+      <c r="O26" t="inlineStr"/>
+      <c r="P26" t="inlineStr"/>
+      <c r="Q26" t="inlineStr"/>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>8609356930</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Dire</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>Rubick</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>Frugal Filch</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr"/>
+      <c r="I27" t="inlineStr">
+        <is>
+          <t>Frugal Filch</t>
+        </is>
+      </c>
+      <c r="J27" t="inlineStr">
+        <is>
+          <t>Frugal Filch</t>
+        </is>
+      </c>
+      <c r="K27" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="L27" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="M27" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="N27" t="inlineStr">
+        <is>
+          <t>4.2k</t>
+        </is>
+      </c>
+      <c r="O27" t="inlineStr"/>
+      <c r="P27" t="inlineStr"/>
+      <c r="Q27" t="inlineStr"/>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>8609356930</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Dire</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>Abaddon</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>The Quickening</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr"/>
+      <c r="I28" t="inlineStr">
+        <is>
+          <t>The Quickening</t>
+        </is>
+      </c>
+      <c r="J28" t="inlineStr">
+        <is>
+          <t>The Quickening</t>
+        </is>
+      </c>
+      <c r="K28" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="L28" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="M28" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="N28" t="inlineStr">
+        <is>
+          <t>3.7k</t>
+        </is>
+      </c>
+      <c r="O28" t="inlineStr"/>
+      <c r="P28" t="inlineStr"/>
+      <c r="Q28" t="inlineStr"/>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>8609356930</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Dire</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>Earthshaker</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>Tectonic Buildup</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>5025</t>
+        </is>
+      </c>
+      <c r="I29" t="inlineStr">
+        <is>
+          <t>Tectonic Buildup</t>
+        </is>
+      </c>
+      <c r="J29" t="inlineStr">
+        <is>
+          <t>Tectonic Buildup</t>
+        </is>
+      </c>
+      <c r="K29" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="L29" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="M29" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="N29" t="inlineStr">
+        <is>
+          <t>7.1k</t>
+        </is>
+      </c>
+      <c r="O29" t="inlineStr"/>
+      <c r="P29" t="inlineStr"/>
+      <c r="Q29" t="inlineStr"/>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>8609356930</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>Dire</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>Riki</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>Cutthroat</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr"/>
+      <c r="I30" t="inlineStr">
+        <is>
+          <t>Cutthroat</t>
+        </is>
+      </c>
+      <c r="J30" t="inlineStr">
+        <is>
+          <t>Cutthroat</t>
+        </is>
+      </c>
+      <c r="K30" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L30" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="M30" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="N30" t="inlineStr">
+        <is>
+          <t>5.4k</t>
+        </is>
+      </c>
+      <c r="O30" t="inlineStr"/>
+      <c r="P30" t="inlineStr"/>
+      <c r="Q30" t="inlineStr"/>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>8609356930</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>Dire</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>Juggernaut</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>Bladeform</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>7021</t>
+        </is>
+      </c>
+      <c r="I31" t="inlineStr">
+        <is>
+          <t>Bladeform</t>
+        </is>
+      </c>
+      <c r="J31" t="inlineStr">
+        <is>
+          <t>Bladeform</t>
+        </is>
+      </c>
+      <c r="K31" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="L31" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="M31" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="N31" t="inlineStr">
+        <is>
+          <t>10.1k</t>
+        </is>
+      </c>
+      <c r="O31" t="inlineStr"/>
+      <c r="P31" t="inlineStr"/>
+      <c r="Q31" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1350,7 +2838,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P11"/>
+  <dimension ref="A1:P21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2250,6 +3738,826 @@
         </is>
       </c>
       <c r="P11" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>8609332493</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Vengeful Spirit</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Проигрыш</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Силы Света</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>Силы Света Слж/Верхняя</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>Сложная</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>Верхняя</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>Сложная</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>3287</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>3321</t>
+        </is>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="M12" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="N12" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="O12" t="inlineStr">
+        <is>
+          <t>28</t>
+        </is>
+      </c>
+      <c r="P12" t="inlineStr">
+        <is>
+          <t>38</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>8609332493</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Skywrath Mage</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Ничья</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Силы Света</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>Силы Света Мид</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>Средняя</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>Центр</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>Средняя</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>5534</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>6395</t>
+        </is>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="L13" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="M13" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="N13" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="O13" t="inlineStr">
+        <is>
+          <t>28</t>
+        </is>
+      </c>
+      <c r="P13" t="inlineStr">
+        <is>
+          <t>51</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>8609332493</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Largo</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Ничья</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Силы Света</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>Силы Света Легкая/Нижняя</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>Легкая</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>Нижняя</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>Легкая</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>2184</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>2417</t>
+        </is>
+      </c>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L14" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="M14" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="N14" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="O14" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="P14" t="inlineStr">
+        <is>
+          <t>14</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>8609332493</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Ursa</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Ничья</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>Силы Света</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>Силы Света Легкая/Нижняя</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>Легкая</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>Нижняя</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>Легкая</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>6093</t>
+        </is>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>4785</t>
+        </is>
+      </c>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="L15" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="M15" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="N15" t="inlineStr">
+        <is>
+          <t>17</t>
+        </is>
+      </c>
+      <c r="O15" t="inlineStr">
+        <is>
+          <t>38</t>
+        </is>
+      </c>
+      <c r="P15" t="inlineStr">
+        <is>
+          <t>75</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>8609332493</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Shadow Shaman</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Проигрыш</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Силы Света</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>Силы Света Роуминг</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>Роуминг</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>Роум</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>Роуминг</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>2570</t>
+        </is>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>3027</t>
+        </is>
+      </c>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="L16" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="M16" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="N16" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="O16" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="P16" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>8609332493</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Drow Ranger</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Выигрыш</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Силы Тьмы</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>Силы Тьмы Легкая/Верхняя</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>Легкая</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>Верхняя</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>Легкая</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>6570</t>
+        </is>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>7440</t>
+        </is>
+      </c>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="L17" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="M17" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="N17" t="inlineStr">
+        <is>
+          <t>13</t>
+        </is>
+      </c>
+      <c r="O17" t="inlineStr">
+        <is>
+          <t>39</t>
+        </is>
+      </c>
+      <c r="P17" t="inlineStr">
+        <is>
+          <t>91</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>8609332493</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Arc Warden</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Ничья</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>Силы Тьмы</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>Силы Тьмы Мид</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>Средняя</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>Центр</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>Средняя</t>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>5258</t>
+        </is>
+      </c>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>5162</t>
+        </is>
+      </c>
+      <c r="K18" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="L18" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="M18" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="N18" t="inlineStr">
+        <is>
+          <t>22</t>
+        </is>
+      </c>
+      <c r="O18" t="inlineStr">
+        <is>
+          <t>39</t>
+        </is>
+      </c>
+      <c r="P18" t="inlineStr">
+        <is>
+          <t>64</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>8609332493</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Lion</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Ничья</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>Силы Тьмы</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>Силы Тьмы Слж/Нижняя</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>Сложная</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>Нижняя</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>Сложная</t>
+        </is>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>1992</t>
+        </is>
+      </c>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>2579</t>
+        </is>
+      </c>
+      <c r="K19" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L19" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="M19" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="N19" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="O19" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="P19" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>8609332493</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Magnus</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Ничья</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>Силы Тьмы</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>Силы Тьмы Слж/Нижняя</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>Сложная</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>Нижняя</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>Сложная</t>
+        </is>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>5602</t>
+        </is>
+      </c>
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>3922</t>
+        </is>
+      </c>
+      <c r="K20" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="L20" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="M20" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="N20" t="inlineStr">
+        <is>
+          <t>27</t>
+        </is>
+      </c>
+      <c r="O20" t="inlineStr">
+        <is>
+          <t>54</t>
+        </is>
+      </c>
+      <c r="P20" t="inlineStr">
+        <is>
+          <t>81</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>8609332493</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Tusk</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Выигрыш</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>Силы Тьмы</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>Силы Тьмы Роуминг</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>Роуминг</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>Роум</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>Роуминг</t>
+        </is>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>2572</t>
+        </is>
+      </c>
+      <c r="J21" t="inlineStr">
+        <is>
+          <t>3046</t>
+        </is>
+      </c>
+      <c r="K21" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="L21" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="M21" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="N21" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="O21" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="P21" t="inlineStr">
         <is>
           <t>2</t>
         </is>
@@ -2266,7 +4574,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O11"/>
+  <dimension ref="A1:O21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3111,6 +5419,776 @@
         </is>
       </c>
       <c r="O11" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>8609332493</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Vengeful Spirit</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Проигрыш</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Силы Света</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>Силы Света Слж/Верхняя</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>Сложная</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>Верхняя</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>3287</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>3321</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="M12" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="N12" t="inlineStr">
+        <is>
+          <t>28</t>
+        </is>
+      </c>
+      <c r="O12" t="inlineStr">
+        <is>
+          <t>38</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>8609332493</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Skywrath Mage</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Ничья</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Силы Света</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>Силы Света Мид</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>Средняя</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>Центр</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>5534</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>6395</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="L13" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="M13" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="N13" t="inlineStr">
+        <is>
+          <t>28</t>
+        </is>
+      </c>
+      <c r="O13" t="inlineStr">
+        <is>
+          <t>51</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>8609332493</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Largo</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Ничья</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Силы Света</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>Силы Света Легкая/Нижняя</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>Легкая</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>Нижняя</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>2184</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>2417</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="L14" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="M14" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="N14" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="O14" t="inlineStr">
+        <is>
+          <t>14</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>8609332493</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Ursa</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Ничья</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>Силы Света</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>Силы Света Легкая/Нижняя</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>Легкая</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>Нижняя</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>6093</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>4785</t>
+        </is>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="L15" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="M15" t="inlineStr">
+        <is>
+          <t>17</t>
+        </is>
+      </c>
+      <c r="N15" t="inlineStr">
+        <is>
+          <t>38</t>
+        </is>
+      </c>
+      <c r="O15" t="inlineStr">
+        <is>
+          <t>75</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>8609332493</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Shadow Shaman</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Проигрыш</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Силы Света</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>Силы Света Роуминг</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>Роуминг</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>Роум</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>2570</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>3027</t>
+        </is>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="L16" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="M16" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="N16" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="O16" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>8609332493</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Drow Ranger</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Выигрыш</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Силы Тьмы</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>Силы Тьмы Легкая/Верхняя</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>Легкая</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>Верхняя</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>6570</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>7440</t>
+        </is>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="L17" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="M17" t="inlineStr">
+        <is>
+          <t>13</t>
+        </is>
+      </c>
+      <c r="N17" t="inlineStr">
+        <is>
+          <t>39</t>
+        </is>
+      </c>
+      <c r="O17" t="inlineStr">
+        <is>
+          <t>91</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>8609332493</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Arc Warden</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Ничья</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>Силы Тьмы</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>Силы Тьмы Мид</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>Средняя</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>Центр</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>5258</t>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>5162</t>
+        </is>
+      </c>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="K18" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="L18" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="M18" t="inlineStr">
+        <is>
+          <t>22</t>
+        </is>
+      </c>
+      <c r="N18" t="inlineStr">
+        <is>
+          <t>39</t>
+        </is>
+      </c>
+      <c r="O18" t="inlineStr">
+        <is>
+          <t>64</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>8609332493</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Lion</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Ничья</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>Силы Тьмы</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>Силы Тьмы Слж/Нижняя</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>Сложная</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>Нижняя</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>1992</t>
+        </is>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>2579</t>
+        </is>
+      </c>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K19" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L19" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="M19" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="N19" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="O19" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>8609332493</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Magnus</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Ничья</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>Силы Тьмы</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>Силы Тьмы Слж/Нижняя</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>Сложная</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>Нижняя</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>5602</t>
+        </is>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>3922</t>
+        </is>
+      </c>
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="K20" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="L20" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="M20" t="inlineStr">
+        <is>
+          <t>27</t>
+        </is>
+      </c>
+      <c r="N20" t="inlineStr">
+        <is>
+          <t>54</t>
+        </is>
+      </c>
+      <c r="O20" t="inlineStr">
+        <is>
+          <t>81</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>8609332493</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Tusk</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Выигрыш</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>Силы Тьмы</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>Силы Тьмы Роуминг</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>Роуминг</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>Роум</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>2572</t>
+        </is>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>3046</t>
+        </is>
+      </c>
+      <c r="J21" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="K21" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="L21" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="M21" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="N21" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="O21" t="inlineStr">
         <is>
           <t>2</t>
         </is>
@@ -3127,7 +6205,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O11"/>
+  <dimension ref="A1:O21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3977,6 +7055,776 @@
         </is>
       </c>
     </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>8609332493</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Vengeful Spirit</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Проигрыш</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Силы Света</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>Силы Света Слж/Верхняя</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>Сложная</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>Верхняя</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>3287</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>3321</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="M12" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="N12" t="inlineStr">
+        <is>
+          <t>28</t>
+        </is>
+      </c>
+      <c r="O12" t="inlineStr">
+        <is>
+          <t>38</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>8609332493</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Skywrath Mage</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Ничья</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Силы Света</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>Силы Света Мид</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>Средняя</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>Центр</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>5534</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>6395</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="L13" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="M13" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="N13" t="inlineStr">
+        <is>
+          <t>28</t>
+        </is>
+      </c>
+      <c r="O13" t="inlineStr">
+        <is>
+          <t>51</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>8609332493</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Largo</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Ничья</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Силы Света</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>Силы Света Легкая/Нижняя</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>Легкая</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>Нижняя</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>2184</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>2417</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="L14" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="M14" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="N14" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="O14" t="inlineStr">
+        <is>
+          <t>14</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>8609332493</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Ursa</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Ничья</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>Силы Света</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>Силы Света Легкая/Нижняя</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>Легкая</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>Нижняя</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>6093</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>4785</t>
+        </is>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="L15" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="M15" t="inlineStr">
+        <is>
+          <t>17</t>
+        </is>
+      </c>
+      <c r="N15" t="inlineStr">
+        <is>
+          <t>38</t>
+        </is>
+      </c>
+      <c r="O15" t="inlineStr">
+        <is>
+          <t>75</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>8609332493</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Shadow Shaman</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Проигрыш</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Силы Света</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>Силы Света Роуминг</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>Роуминг</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>Роум</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>2570</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>3027</t>
+        </is>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="L16" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="M16" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="N16" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="O16" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>8609332493</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Drow Ranger</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Выигрыш</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Силы Тьмы</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>Силы Тьмы Легкая/Верхняя</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>Легкая</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>Верхняя</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>6570</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>7440</t>
+        </is>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="L17" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="M17" t="inlineStr">
+        <is>
+          <t>13</t>
+        </is>
+      </c>
+      <c r="N17" t="inlineStr">
+        <is>
+          <t>39</t>
+        </is>
+      </c>
+      <c r="O17" t="inlineStr">
+        <is>
+          <t>91</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>8609332493</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Arc Warden</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Ничья</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>Силы Тьмы</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>Силы Тьмы Мид</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>Средняя</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>Центр</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>5258</t>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>5162</t>
+        </is>
+      </c>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="K18" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="L18" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="M18" t="inlineStr">
+        <is>
+          <t>22</t>
+        </is>
+      </c>
+      <c r="N18" t="inlineStr">
+        <is>
+          <t>39</t>
+        </is>
+      </c>
+      <c r="O18" t="inlineStr">
+        <is>
+          <t>64</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>8609332493</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Lion</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Ничья</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>Силы Тьмы</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>Силы Тьмы Слж/Нижняя</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>Сложная</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>Нижняя</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>1992</t>
+        </is>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>2579</t>
+        </is>
+      </c>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K19" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L19" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="M19" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="N19" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="O19" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>8609332493</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Magnus</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Ничья</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>Силы Тьмы</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>Силы Тьмы Слж/Нижняя</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>Сложная</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>Нижняя</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>5602</t>
+        </is>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>3922</t>
+        </is>
+      </c>
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="K20" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="L20" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="M20" t="inlineStr">
+        <is>
+          <t>27</t>
+        </is>
+      </c>
+      <c r="N20" t="inlineStr">
+        <is>
+          <t>54</t>
+        </is>
+      </c>
+      <c r="O20" t="inlineStr">
+        <is>
+          <t>81</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>8609332493</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Tusk</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Выигрыш</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>Силы Тьмы</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>Силы Тьмы Роуминг</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>Роуминг</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>Роум</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>2572</t>
+        </is>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>3046</t>
+        </is>
+      </c>
+      <c r="J21" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="K21" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="L21" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="M21" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="N21" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="O21" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>